<commit_message>
feat: takeout email required validation
</commit_message>
<xml_diff>
--- a/public/template_excel/DATA PEGAWAI NON ASN.xlsx
+++ b/public/template_excel/DATA PEGAWAI NON ASN.xlsx
@@ -630,9 +630,6 @@
     <t>Alamat Sesuai KTP</t>
   </si>
   <si>
-    <t>Email *</t>
-  </si>
-  <si>
     <t>Jenis Perbantuan *</t>
   </si>
   <si>
@@ -658,6 +655,9 @@
   </si>
   <si>
     <t xml:space="preserve">TMT Jabatan </t>
+  </si>
+  <si>
+    <t>Email</t>
   </si>
 </sst>
 </file>
@@ -1090,7 +1090,7 @@
         <v>36</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="L1" s="2" t="s">
         <v>37</v>
@@ -1117,7 +1117,7 @@
         <v>39</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="U1" s="2" t="s">
         <v>40</v>
@@ -1129,7 +1129,7 @@
         <v>5</v>
       </c>
       <c r="X1" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="Y1" s="2" t="s">
         <v>42</v>
@@ -1156,13 +1156,13 @@
         <v>10</v>
       </c>
       <c r="AG1" s="2" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="AH1" s="2" t="s">
         <v>34</v>
       </c>
       <c r="AI1" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:35" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -1202,13 +1202,13 @@
   <sheetData>
     <row r="1" spans="1:19" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>50</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>51</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>23</v>
@@ -1217,7 +1217,7 @@
         <v>35</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>11</v>
@@ -1229,7 +1229,7 @@
         <v>13</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>14</v>

</xml_diff>